<commit_message>
CHANGED SOME THINGS AND ADDED SOME STOCK
</commit_message>
<xml_diff>
--- a/frontend/public/templates/pharmacy_import_template.xlsx
+++ b/frontend/public/templates/pharmacy_import_template.xlsx
@@ -399,8 +399,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:W107"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="1" max="1" width="27.83203125" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" customWidth="1"/>
     <col min="3" max="3" width="14.83203125" customWidth="1"/>
     <col min="4" max="4" width="21.83203125" customWidth="1"/>
     <col min="5" max="5" width="21.83203125" customWidth="1"/>
@@ -414,7 +414,7 @@
     <col min="13" max="13" width="12.83203125" customWidth="1"/>
     <col min="14" max="14" width="17.83203125" customWidth="1"/>
     <col min="15" max="15" width="21.83203125" customWidth="1"/>
-    <col min="16" max="16" width="25.83203125" customWidth="1"/>
+    <col min="16" max="16" width="34.83203125" customWidth="1"/>
     <col min="17" max="17" width="17.83203125" customWidth="1"/>
     <col min="18" max="18" width="14.83203125" customWidth="1"/>
     <col min="19" max="19" width="14.83203125" customWidth="1"/>
@@ -426,25 +426,25 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>MediCore Pharmacy Stock Import - Supplier Purchase Bill</v>
+        <v>MediCore Pharmacy Stock Import - Current Stock</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Medicine Name may be blank when Brand Name is available. Form accepts any text. Supplier, rack location, and base unit are not required.</v>
+        <v>Medicine Name and Batch Number are optional. Brand Name can be used. Blank names become Imported Medicine row no.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Required: Medicine or Brand, Batch, Expiry, Qty, MRP, Selling Price, GST. Dates should be YYYY-MM-DD.</v>
+        <v>Required: Expiry, Qty, MRP, Selling Price, GST. Supplier, rack location, and base unit are not required.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Medicine Name</v>
+        <v>Medicine Name (Optional)</v>
       </c>
       <c r="B4" t="str">
-        <v>Batch Number</v>
+        <v>Batch Number (Optional)</v>
       </c>
       <c r="C4" t="str">
         <v>Expiry Date</v>
@@ -486,7 +486,7 @@
         <v>Manufacturing Date</v>
       </c>
       <c r="P4" t="str">
-        <v>Purchase Rate Per Pack</v>
+        <v>Purchase Rate Per Pack (Optional)</v>
       </c>
       <c r="Q4" t="str">
         <v>Taxable Amount</v>
@@ -512,10 +512,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Paracetamol</v>
+        <v/>
       </c>
       <c r="B5" t="str">
-        <v>DL500-A1</v>
+        <v/>
       </c>
       <c r="C5" t="str">
         <v>2028-12-31</v>
@@ -551,13 +551,13 @@
         <v>strip</v>
       </c>
       <c r="N5">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="O5" t="str">
-        <v>2026-01-01</v>
-      </c>
-      <c r="P5">
-        <v>215</v>
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v/>
       </c>
       <c r="Q5">
         <f>IF(OR(D5=0,P5=0),0,ROUND((D5+(E5/MAX(1,N5)))*P5,2))</f>
@@ -587,10 +587,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Amoxicillin</v>
+        <v/>
       </c>
       <c r="B6" t="str">
-        <v>NM500-B1</v>
+        <v/>
       </c>
       <c r="C6" t="str">
         <v>2028-08-31</v>
@@ -629,10 +629,10 @@
         <v>10</v>
       </c>
       <c r="O6" t="str">
-        <v>2026-02-01</v>
-      </c>
-      <c r="P6">
-        <v>820</v>
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v/>
       </c>
       <c r="Q6">
         <f>IF(OR(D6=0,P6=0),0,ROUND((D6+(E6/MAX(1,N6)))*P6,2))</f>
@@ -662,10 +662,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Insulin Human</v>
+        <v/>
       </c>
       <c r="B7" t="str">
-        <v>HIN40-C1</v>
+        <v/>
       </c>
       <c r="C7" t="str">
         <v>2027-06-30</v>
@@ -704,10 +704,10 @@
         <v>1</v>
       </c>
       <c r="O7" t="str">
-        <v>2026-03-01</v>
-      </c>
-      <c r="P7">
-        <v>118</v>
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v/>
       </c>
       <c r="Q7">
         <f>IF(OR(D7=0,P7=0),0,ROUND((D7+(E7/MAX(1,N7)))*P7,2))</f>

</xml_diff>